<commit_message>
feature of family group y feature test
</commit_message>
<xml_diff>
--- a/database/seeders/database.xlsx
+++ b/database/seeders/database.xlsx
@@ -1,22 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29725"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\wamp64\www\cocoo-nova\database\seeders\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CC10ED45-77CD-475D-A12D-689F75CB76D2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7559695F-8A67-482F-AFC3-0AFA7B7166A8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-23148" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
+    <sheet name="humantalent_employees" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Hoja1!$A$1:$AD$251</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">humantalent_employees!$A$1:$AF$251</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4895" uniqueCount="1205">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4897" uniqueCount="1207">
   <si>
     <t>type_document</t>
   </si>
@@ -3654,6 +3654,12 @@
   </si>
   <si>
     <t>REVISAR</t>
+  </si>
+  <si>
+    <t>status</t>
+  </si>
+  <si>
+    <t>photo_path</t>
   </si>
 </sst>
 </file>
@@ -3976,40 +3982,41 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AD251"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <dimension ref="A1:AF251"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.77734375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="13.90625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="11.7265625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="20.6328125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="13.453125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="20.08984375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="13.88671875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="11.77734375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="20.6640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="13.44140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="20.109375" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="24" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="52.90625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="14.453125" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="53.08984375" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="6.7265625" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="13.54296875" customWidth="1"/>
-    <col min="12" max="12" width="12.54296875" customWidth="1"/>
-    <col min="13" max="13" width="10.7265625" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="24.90625" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="6.6328125" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="10.08984375" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="15.7265625" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="27.453125" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="10.26953125" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="12.7265625" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="15.1796875" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="13.81640625" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="11.453125" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="19.08984375" bestFit="1" customWidth="1"/>
-    <col min="25" max="25" width="52.453125" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="32.26953125" bestFit="1" customWidth="1"/>
-    <col min="27" max="27" width="12.7265625" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="8.81640625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="52.88671875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="14.44140625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="53.109375" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="6.77734375" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="13.5546875" customWidth="1"/>
+    <col min="12" max="12" width="12.5546875" customWidth="1"/>
+    <col min="13" max="13" width="10.77734375" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="24.88671875" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="6.6640625" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="10.109375" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="15.77734375" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="27.44140625" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="10.21875" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="12.77734375" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="15.21875" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="13.77734375" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="11.44140625" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="19.109375" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="52.44140625" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="32.21875" bestFit="1" customWidth="1"/>
+    <col min="27" max="27" width="12.77734375" bestFit="1" customWidth="1"/>
+    <col min="28" max="28" width="8.77734375" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="10.5546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -4100,8 +4107,14 @@
       <c r="AD1" t="s">
         <v>29</v>
       </c>
+      <c r="AE1" t="s">
+        <v>1206</v>
+      </c>
+      <c r="AF1" t="s">
+        <v>1205</v>
+      </c>
     </row>
-    <row r="2" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>30</v>
       </c>
@@ -4192,8 +4205,11 @@
       <c r="AD2">
         <v>0</v>
       </c>
+      <c r="AF2">
+        <v>0</v>
+      </c>
     </row>
-    <row r="3" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>30</v>
       </c>
@@ -4281,8 +4297,11 @@
       <c r="AD3">
         <v>0</v>
       </c>
+      <c r="AF3">
+        <v>1</v>
+      </c>
     </row>
-    <row r="4" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>30</v>
       </c>
@@ -4370,8 +4389,11 @@
       <c r="AD4">
         <v>0</v>
       </c>
+      <c r="AF4">
+        <v>0</v>
+      </c>
     </row>
-    <row r="5" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>30</v>
       </c>
@@ -4459,8 +4481,11 @@
       <c r="AD5">
         <v>0</v>
       </c>
+      <c r="AF5">
+        <v>1</v>
+      </c>
     </row>
-    <row r="6" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>30</v>
       </c>
@@ -4548,8 +4573,11 @@
       <c r="AD6">
         <v>0</v>
       </c>
+      <c r="AF6">
+        <v>1</v>
+      </c>
     </row>
-    <row r="7" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>30</v>
       </c>
@@ -4640,8 +4668,11 @@
       <c r="AD7">
         <v>0</v>
       </c>
+      <c r="AF7">
+        <v>1</v>
+      </c>
     </row>
-    <row r="8" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>30</v>
       </c>
@@ -4732,8 +4763,11 @@
       <c r="AD8">
         <v>0</v>
       </c>
+      <c r="AF8">
+        <v>0</v>
+      </c>
     </row>
-    <row r="9" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>30</v>
       </c>
@@ -4824,8 +4858,11 @@
       <c r="AD9">
         <v>0</v>
       </c>
+      <c r="AF9">
+        <v>0</v>
+      </c>
     </row>
-    <row r="10" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>30</v>
       </c>
@@ -4913,8 +4950,11 @@
       <c r="AD10">
         <v>0</v>
       </c>
+      <c r="AF10">
+        <v>0</v>
+      </c>
     </row>
-    <row r="11" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>30</v>
       </c>
@@ -5002,8 +5042,11 @@
       <c r="AD11">
         <v>0</v>
       </c>
+      <c r="AF11">
+        <v>0</v>
+      </c>
     </row>
-    <row r="12" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>30</v>
       </c>
@@ -5091,8 +5134,11 @@
       <c r="AD12">
         <v>0</v>
       </c>
+      <c r="AF12">
+        <v>1</v>
+      </c>
     </row>
-    <row r="13" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>30</v>
       </c>
@@ -5180,8 +5226,11 @@
       <c r="AD13">
         <v>0</v>
       </c>
+      <c r="AF13">
+        <v>1</v>
+      </c>
     </row>
-    <row r="14" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>30</v>
       </c>
@@ -5269,8 +5318,11 @@
       <c r="AD14">
         <v>0</v>
       </c>
+      <c r="AF14">
+        <v>0</v>
+      </c>
     </row>
-    <row r="15" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>30</v>
       </c>
@@ -5358,8 +5410,11 @@
       <c r="AD15">
         <v>0</v>
       </c>
+      <c r="AF15">
+        <v>0</v>
+      </c>
     </row>
-    <row r="16" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>30</v>
       </c>
@@ -5447,8 +5502,11 @@
       <c r="AD16">
         <v>0</v>
       </c>
+      <c r="AF16">
+        <v>0</v>
+      </c>
     </row>
-    <row r="17" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>30</v>
       </c>
@@ -5536,8 +5594,11 @@
       <c r="AD17">
         <v>0</v>
       </c>
+      <c r="AF17">
+        <v>1</v>
+      </c>
     </row>
-    <row r="18" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>30</v>
       </c>
@@ -5625,8 +5686,11 @@
       <c r="AD18">
         <v>0</v>
       </c>
+      <c r="AF18">
+        <v>1</v>
+      </c>
     </row>
-    <row r="19" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>30</v>
       </c>
@@ -5714,8 +5778,11 @@
       <c r="AD19">
         <v>0</v>
       </c>
+      <c r="AF19">
+        <v>1</v>
+      </c>
     </row>
-    <row r="20" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>30</v>
       </c>
@@ -5803,8 +5870,11 @@
       <c r="AD20">
         <v>0</v>
       </c>
+      <c r="AF20">
+        <v>0</v>
+      </c>
     </row>
-    <row r="21" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
         <v>30</v>
       </c>
@@ -5892,8 +5962,11 @@
       <c r="AD21">
         <v>0</v>
       </c>
+      <c r="AF21">
+        <v>1</v>
+      </c>
     </row>
-    <row r="22" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
         <v>30</v>
       </c>
@@ -5981,8 +6054,11 @@
       <c r="AD22">
         <v>0</v>
       </c>
+      <c r="AF22">
+        <v>1</v>
+      </c>
     </row>
-    <row r="23" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
         <v>30</v>
       </c>
@@ -6070,8 +6146,11 @@
       <c r="AD23">
         <v>0</v>
       </c>
+      <c r="AF23">
+        <v>0</v>
+      </c>
     </row>
-    <row r="24" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
         <v>30</v>
       </c>
@@ -6159,8 +6238,11 @@
       <c r="AD24">
         <v>0</v>
       </c>
+      <c r="AF24">
+        <v>1</v>
+      </c>
     </row>
-    <row r="25" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
         <v>30</v>
       </c>
@@ -6248,8 +6330,11 @@
       <c r="AD25">
         <v>0</v>
       </c>
+      <c r="AF25">
+        <v>0</v>
+      </c>
     </row>
-    <row r="26" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
         <v>30</v>
       </c>
@@ -6337,8 +6422,11 @@
       <c r="AD26">
         <v>0</v>
       </c>
+      <c r="AF26">
+        <v>0</v>
+      </c>
     </row>
-    <row r="27" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
         <v>30</v>
       </c>
@@ -6426,8 +6514,11 @@
       <c r="AD27">
         <v>0</v>
       </c>
+      <c r="AF27">
+        <v>0</v>
+      </c>
     </row>
-    <row r="28" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
         <v>30</v>
       </c>
@@ -6515,8 +6606,11 @@
       <c r="AD28">
         <v>0</v>
       </c>
+      <c r="AF28">
+        <v>1</v>
+      </c>
     </row>
-    <row r="29" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
         <v>30</v>
       </c>
@@ -6604,8 +6698,11 @@
       <c r="AD29">
         <v>0</v>
       </c>
+      <c r="AF29">
+        <v>0</v>
+      </c>
     </row>
-    <row r="30" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
         <v>30</v>
       </c>
@@ -6693,8 +6790,11 @@
       <c r="AD30">
         <v>0</v>
       </c>
+      <c r="AF30">
+        <v>1</v>
+      </c>
     </row>
-    <row r="31" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
         <v>30</v>
       </c>
@@ -6782,8 +6882,11 @@
       <c r="AD31">
         <v>0</v>
       </c>
+      <c r="AF31">
+        <v>1</v>
+      </c>
     </row>
-    <row r="32" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
         <v>30</v>
       </c>
@@ -6871,8 +6974,11 @@
       <c r="AD32">
         <v>0</v>
       </c>
+      <c r="AF32">
+        <v>0</v>
+      </c>
     </row>
-    <row r="33" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
         <v>30</v>
       </c>
@@ -6960,8 +7066,11 @@
       <c r="AD33">
         <v>0</v>
       </c>
+      <c r="AF33">
+        <v>0</v>
+      </c>
     </row>
-    <row r="34" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
         <v>30</v>
       </c>
@@ -7049,8 +7158,11 @@
       <c r="AD34">
         <v>0</v>
       </c>
+      <c r="AF34">
+        <v>0</v>
+      </c>
     </row>
-    <row r="35" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
         <v>30</v>
       </c>
@@ -7138,8 +7250,11 @@
       <c r="AD35">
         <v>0</v>
       </c>
+      <c r="AF35">
+        <v>0</v>
+      </c>
     </row>
-    <row r="36" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
         <v>30</v>
       </c>
@@ -7227,8 +7342,11 @@
       <c r="AD36">
         <v>0</v>
       </c>
+      <c r="AF36">
+        <v>0</v>
+      </c>
     </row>
-    <row r="37" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
         <v>30</v>
       </c>
@@ -7319,8 +7437,11 @@
       <c r="AD37">
         <v>0</v>
       </c>
+      <c r="AF37">
+        <v>1</v>
+      </c>
     </row>
-    <row r="38" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
         <v>30</v>
       </c>
@@ -7408,8 +7529,11 @@
       <c r="AD38">
         <v>0</v>
       </c>
+      <c r="AF38">
+        <v>0</v>
+      </c>
     </row>
-    <row r="39" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
         <v>30</v>
       </c>
@@ -7497,8 +7621,11 @@
       <c r="AD39">
         <v>0</v>
       </c>
+      <c r="AF39">
+        <v>0</v>
+      </c>
     </row>
-    <row r="40" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
         <v>30</v>
       </c>
@@ -7586,8 +7713,11 @@
       <c r="AD40">
         <v>0</v>
       </c>
+      <c r="AF40">
+        <v>1</v>
+      </c>
     </row>
-    <row r="41" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
         <v>30</v>
       </c>
@@ -7675,8 +7805,11 @@
       <c r="AD41">
         <v>0</v>
       </c>
+      <c r="AF41">
+        <v>0</v>
+      </c>
     </row>
-    <row r="42" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
         <v>30</v>
       </c>
@@ -7764,8 +7897,11 @@
       <c r="AD42">
         <v>0</v>
       </c>
+      <c r="AF42">
+        <v>0</v>
+      </c>
     </row>
-    <row r="43" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
         <v>30</v>
       </c>
@@ -7853,8 +7989,11 @@
       <c r="AD43">
         <v>0</v>
       </c>
+      <c r="AF43">
+        <v>0</v>
+      </c>
     </row>
-    <row r="44" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A44" t="s">
         <v>30</v>
       </c>
@@ -7942,8 +8081,11 @@
       <c r="AD44">
         <v>0</v>
       </c>
+      <c r="AF44">
+        <v>0</v>
+      </c>
     </row>
-    <row r="45" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A45" t="s">
         <v>30</v>
       </c>
@@ -8031,8 +8173,11 @@
       <c r="AD45">
         <v>0</v>
       </c>
+      <c r="AF45">
+        <v>0</v>
+      </c>
     </row>
-    <row r="46" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A46" t="s">
         <v>30</v>
       </c>
@@ -8120,8 +8265,11 @@
       <c r="AD46">
         <v>0</v>
       </c>
+      <c r="AF46">
+        <v>0</v>
+      </c>
     </row>
-    <row r="47" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A47" t="s">
         <v>30</v>
       </c>
@@ -8212,8 +8360,11 @@
       <c r="AD47">
         <v>0</v>
       </c>
+      <c r="AF47">
+        <v>1</v>
+      </c>
     </row>
-    <row r="48" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A48" t="s">
         <v>30</v>
       </c>
@@ -8301,8 +8452,11 @@
       <c r="AD48">
         <v>0</v>
       </c>
+      <c r="AF48">
+        <v>1</v>
+      </c>
     </row>
-    <row r="49" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A49" t="s">
         <v>30</v>
       </c>
@@ -8390,8 +8544,11 @@
       <c r="AD49">
         <v>0</v>
       </c>
+      <c r="AF49">
+        <v>0</v>
+      </c>
     </row>
-    <row r="50" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A50" t="s">
         <v>30</v>
       </c>
@@ -8482,8 +8639,11 @@
       <c r="AD50">
         <v>0</v>
       </c>
+      <c r="AF50">
+        <v>0</v>
+      </c>
     </row>
-    <row r="51" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A51" t="s">
         <v>30</v>
       </c>
@@ -8571,8 +8731,11 @@
       <c r="AD51">
         <v>0</v>
       </c>
+      <c r="AF51">
+        <v>0</v>
+      </c>
     </row>
-    <row r="52" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A52" t="s">
         <v>30</v>
       </c>
@@ -8660,8 +8823,11 @@
       <c r="AD52">
         <v>0</v>
       </c>
+      <c r="AF52">
+        <v>0</v>
+      </c>
     </row>
-    <row r="53" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A53" t="s">
         <v>30</v>
       </c>
@@ -8749,8 +8915,11 @@
       <c r="AD53">
         <v>0</v>
       </c>
+      <c r="AF53">
+        <v>0</v>
+      </c>
     </row>
-    <row r="54" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A54" t="s">
         <v>30</v>
       </c>
@@ -8838,8 +9007,11 @@
       <c r="AD54">
         <v>0</v>
       </c>
+      <c r="AF54">
+        <v>0</v>
+      </c>
     </row>
-    <row r="55" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A55" t="s">
         <v>30</v>
       </c>
@@ -8927,8 +9099,11 @@
       <c r="AD55">
         <v>0</v>
       </c>
+      <c r="AF55">
+        <v>0</v>
+      </c>
     </row>
-    <row r="56" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A56" t="s">
         <v>30</v>
       </c>
@@ -9016,8 +9191,11 @@
       <c r="AD56">
         <v>0</v>
       </c>
+      <c r="AF56">
+        <v>1</v>
+      </c>
     </row>
-    <row r="57" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A57" t="s">
         <v>30</v>
       </c>
@@ -9105,8 +9283,11 @@
       <c r="AD57">
         <v>0</v>
       </c>
+      <c r="AF57">
+        <v>0</v>
+      </c>
     </row>
-    <row r="58" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A58" t="s">
         <v>30</v>
       </c>
@@ -9197,8 +9378,11 @@
       <c r="AD58">
         <v>0</v>
       </c>
+      <c r="AF58">
+        <v>0</v>
+      </c>
     </row>
-    <row r="59" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A59" t="s">
         <v>30</v>
       </c>
@@ -9286,8 +9470,11 @@
       <c r="AD59">
         <v>0</v>
       </c>
+      <c r="AF59">
+        <v>0</v>
+      </c>
     </row>
-    <row r="60" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A60" t="s">
         <v>30</v>
       </c>
@@ -9375,8 +9562,11 @@
       <c r="AD60">
         <v>0</v>
       </c>
+      <c r="AF60">
+        <v>0</v>
+      </c>
     </row>
-    <row r="61" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A61" t="s">
         <v>30</v>
       </c>
@@ -9464,8 +9654,11 @@
       <c r="AD61">
         <v>0</v>
       </c>
+      <c r="AF61">
+        <v>0</v>
+      </c>
     </row>
-    <row r="62" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A62" t="s">
         <v>30</v>
       </c>
@@ -9553,8 +9746,11 @@
       <c r="AD62">
         <v>0</v>
       </c>
+      <c r="AF62">
+        <v>0</v>
+      </c>
     </row>
-    <row r="63" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A63" t="s">
         <v>30</v>
       </c>
@@ -9642,8 +9838,11 @@
       <c r="AD63">
         <v>0</v>
       </c>
+      <c r="AF63">
+        <v>0</v>
+      </c>
     </row>
-    <row r="64" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A64" t="s">
         <v>30</v>
       </c>
@@ -9731,8 +9930,11 @@
       <c r="AD64">
         <v>0</v>
       </c>
+      <c r="AF64">
+        <v>0</v>
+      </c>
     </row>
-    <row r="65" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A65" t="s">
         <v>30</v>
       </c>
@@ -9820,8 +10022,11 @@
       <c r="AD65">
         <v>0</v>
       </c>
+      <c r="AF65">
+        <v>0</v>
+      </c>
     </row>
-    <row r="66" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="66" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A66" t="s">
         <v>30</v>
       </c>
@@ -9912,8 +10117,11 @@
       <c r="AD66">
         <v>0</v>
       </c>
+      <c r="AF66">
+        <v>0</v>
+      </c>
     </row>
-    <row r="67" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="67" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A67" t="s">
         <v>30</v>
       </c>
@@ -10001,8 +10209,11 @@
       <c r="AD67">
         <v>0</v>
       </c>
+      <c r="AF67">
+        <v>0</v>
+      </c>
     </row>
-    <row r="68" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="68" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A68" t="s">
         <v>30</v>
       </c>
@@ -10090,8 +10301,11 @@
       <c r="AD68">
         <v>0</v>
       </c>
+      <c r="AF68">
+        <v>1</v>
+      </c>
     </row>
-    <row r="69" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="69" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A69" t="s">
         <v>30</v>
       </c>
@@ -10179,8 +10393,11 @@
       <c r="AD69">
         <v>0</v>
       </c>
+      <c r="AF69">
+        <v>0</v>
+      </c>
     </row>
-    <row r="70" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="70" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A70" t="s">
         <v>30</v>
       </c>
@@ -10268,8 +10485,11 @@
       <c r="AD70">
         <v>0</v>
       </c>
+      <c r="AF70">
+        <v>0</v>
+      </c>
     </row>
-    <row r="71" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="71" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A71" t="s">
         <v>30</v>
       </c>
@@ -10351,8 +10571,11 @@
       <c r="AD71">
         <v>0</v>
       </c>
+      <c r="AF71">
+        <v>1</v>
+      </c>
     </row>
-    <row r="72" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="72" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A72" t="s">
         <v>30</v>
       </c>
@@ -10440,8 +10663,11 @@
       <c r="AD72">
         <v>0</v>
       </c>
+      <c r="AF72">
+        <v>0</v>
+      </c>
     </row>
-    <row r="73" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="73" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A73" t="s">
         <v>30</v>
       </c>
@@ -10529,8 +10755,11 @@
       <c r="AD73">
         <v>0</v>
       </c>
+      <c r="AF73">
+        <v>0</v>
+      </c>
     </row>
-    <row r="74" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="74" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A74" t="s">
         <v>30</v>
       </c>
@@ -10618,8 +10847,11 @@
       <c r="AD74">
         <v>0</v>
       </c>
+      <c r="AF74">
+        <v>0</v>
+      </c>
     </row>
-    <row r="75" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="75" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A75" t="s">
         <v>30</v>
       </c>
@@ -10707,8 +10939,11 @@
       <c r="AD75">
         <v>0</v>
       </c>
+      <c r="AF75">
+        <v>0</v>
+      </c>
     </row>
-    <row r="76" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="76" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A76" t="s">
         <v>30</v>
       </c>
@@ -10796,8 +11031,11 @@
       <c r="AD76">
         <v>0</v>
       </c>
+      <c r="AF76">
+        <v>0</v>
+      </c>
     </row>
-    <row r="77" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="77" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A77" t="s">
         <v>30</v>
       </c>
@@ -10885,8 +11123,11 @@
       <c r="AD77">
         <v>0</v>
       </c>
+      <c r="AF77">
+        <v>0</v>
+      </c>
     </row>
-    <row r="78" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="78" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A78" t="s">
         <v>30</v>
       </c>
@@ -10974,8 +11215,11 @@
       <c r="AD78">
         <v>0</v>
       </c>
+      <c r="AF78">
+        <v>0</v>
+      </c>
     </row>
-    <row r="79" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="79" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A79" t="s">
         <v>30</v>
       </c>
@@ -11063,8 +11307,11 @@
       <c r="AD79">
         <v>0</v>
       </c>
+      <c r="AF79">
+        <v>0</v>
+      </c>
     </row>
-    <row r="80" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="80" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A80" t="s">
         <v>30</v>
       </c>
@@ -11152,8 +11399,11 @@
       <c r="AD80">
         <v>0</v>
       </c>
+      <c r="AF80">
+        <v>0</v>
+      </c>
     </row>
-    <row r="81" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="81" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A81" t="s">
         <v>30</v>
       </c>
@@ -11241,8 +11491,11 @@
       <c r="AD81">
         <v>0</v>
       </c>
+      <c r="AF81">
+        <v>0</v>
+      </c>
     </row>
-    <row r="82" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="82" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A82" t="s">
         <v>30</v>
       </c>
@@ -11330,8 +11583,11 @@
       <c r="AD82">
         <v>0</v>
       </c>
+      <c r="AF82">
+        <v>0</v>
+      </c>
     </row>
-    <row r="83" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="83" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A83" t="s">
         <v>30</v>
       </c>
@@ -11419,8 +11675,11 @@
       <c r="AD83">
         <v>0</v>
       </c>
+      <c r="AF83">
+        <v>0</v>
+      </c>
     </row>
-    <row r="84" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="84" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A84" t="s">
         <v>30</v>
       </c>
@@ -11508,8 +11767,11 @@
       <c r="AD84">
         <v>0</v>
       </c>
+      <c r="AF84">
+        <v>0</v>
+      </c>
     </row>
-    <row r="85" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="85" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A85" t="s">
         <v>30</v>
       </c>
@@ -11597,8 +11859,11 @@
       <c r="AD85">
         <v>0</v>
       </c>
+      <c r="AF85">
+        <v>0</v>
+      </c>
     </row>
-    <row r="86" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="86" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A86" t="s">
         <v>30</v>
       </c>
@@ -11686,8 +11951,11 @@
       <c r="AD86">
         <v>0</v>
       </c>
+      <c r="AF86">
+        <v>0</v>
+      </c>
     </row>
-    <row r="87" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="87" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A87" t="s">
         <v>30</v>
       </c>
@@ -11775,8 +12043,11 @@
       <c r="AD87">
         <v>0</v>
       </c>
+      <c r="AF87">
+        <v>0</v>
+      </c>
     </row>
-    <row r="88" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="88" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A88" t="s">
         <v>30</v>
       </c>
@@ -11864,8 +12135,11 @@
       <c r="AD88">
         <v>0</v>
       </c>
+      <c r="AF88">
+        <v>1</v>
+      </c>
     </row>
-    <row r="89" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="89" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A89" t="s">
         <v>30</v>
       </c>
@@ -11953,8 +12227,11 @@
       <c r="AD89">
         <v>0</v>
       </c>
+      <c r="AF89">
+        <v>0</v>
+      </c>
     </row>
-    <row r="90" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="90" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A90" t="s">
         <v>30</v>
       </c>
@@ -12042,8 +12319,11 @@
       <c r="AD90">
         <v>0</v>
       </c>
+      <c r="AF90">
+        <v>0</v>
+      </c>
     </row>
-    <row r="91" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="91" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A91" t="s">
         <v>30</v>
       </c>
@@ -12131,8 +12411,11 @@
       <c r="AD91">
         <v>0</v>
       </c>
+      <c r="AF91">
+        <v>0</v>
+      </c>
     </row>
-    <row r="92" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="92" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A92" t="s">
         <v>30</v>
       </c>
@@ -12220,8 +12503,11 @@
       <c r="AD92">
         <v>0</v>
       </c>
+      <c r="AF92">
+        <v>0</v>
+      </c>
     </row>
-    <row r="93" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="93" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A93" t="s">
         <v>30</v>
       </c>
@@ -12312,8 +12598,11 @@
       <c r="AD93">
         <v>0</v>
       </c>
+      <c r="AF93">
+        <v>1</v>
+      </c>
     </row>
-    <row r="94" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="94" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A94" t="s">
         <v>30</v>
       </c>
@@ -12404,8 +12693,11 @@
       <c r="AD94">
         <v>0</v>
       </c>
+      <c r="AF94">
+        <v>0</v>
+      </c>
     </row>
-    <row r="95" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="95" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A95" t="s">
         <v>30</v>
       </c>
@@ -12493,8 +12785,11 @@
       <c r="AD95">
         <v>0</v>
       </c>
+      <c r="AF95">
+        <v>0</v>
+      </c>
     </row>
-    <row r="96" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="96" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A96" t="s">
         <v>30</v>
       </c>
@@ -12582,8 +12877,11 @@
       <c r="AD96">
         <v>0</v>
       </c>
+      <c r="AF96">
+        <v>0</v>
+      </c>
     </row>
-    <row r="97" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="97" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A97" t="s">
         <v>30</v>
       </c>
@@ -12674,8 +12972,11 @@
       <c r="AD97">
         <v>0</v>
       </c>
+      <c r="AF97">
+        <v>0</v>
+      </c>
     </row>
-    <row r="98" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="98" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A98" t="s">
         <v>30</v>
       </c>
@@ -12763,8 +13064,11 @@
       <c r="AD98">
         <v>0</v>
       </c>
+      <c r="AF98">
+        <v>0</v>
+      </c>
     </row>
-    <row r="99" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="99" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A99" t="s">
         <v>30</v>
       </c>
@@ -12852,8 +13156,11 @@
       <c r="AD99">
         <v>0</v>
       </c>
+      <c r="AF99">
+        <v>0</v>
+      </c>
     </row>
-    <row r="100" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="100" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A100" t="s">
         <v>30</v>
       </c>
@@ -12944,8 +13251,11 @@
       <c r="AD100">
         <v>0</v>
       </c>
+      <c r="AF100">
+        <v>1</v>
+      </c>
     </row>
-    <row r="101" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="101" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A101" t="s">
         <v>30</v>
       </c>
@@ -13033,8 +13343,11 @@
       <c r="AD101">
         <v>0</v>
       </c>
+      <c r="AF101">
+        <v>0</v>
+      </c>
     </row>
-    <row r="102" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="102" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A102" t="s">
         <v>30</v>
       </c>
@@ -13122,8 +13435,11 @@
       <c r="AD102">
         <v>0</v>
       </c>
+      <c r="AF102">
+        <v>0</v>
+      </c>
     </row>
-    <row r="103" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="103" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A103" t="s">
         <v>30</v>
       </c>
@@ -13214,8 +13530,11 @@
       <c r="AD103">
         <v>0</v>
       </c>
+      <c r="AF103">
+        <v>0</v>
+      </c>
     </row>
-    <row r="104" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="104" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A104" t="s">
         <v>30</v>
       </c>
@@ -13306,8 +13625,11 @@
       <c r="AD104">
         <v>0</v>
       </c>
+      <c r="AF104">
+        <v>0</v>
+      </c>
     </row>
-    <row r="105" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="105" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A105" t="s">
         <v>30</v>
       </c>
@@ -13395,8 +13717,11 @@
       <c r="AD105">
         <v>0</v>
       </c>
+      <c r="AF105">
+        <v>0</v>
+      </c>
     </row>
-    <row r="106" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="106" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A106" t="s">
         <v>30</v>
       </c>
@@ -13487,8 +13812,11 @@
       <c r="AD106">
         <v>0</v>
       </c>
+      <c r="AF106">
+        <v>1</v>
+      </c>
     </row>
-    <row r="107" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="107" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A107" t="s">
         <v>30</v>
       </c>
@@ -13576,8 +13904,11 @@
       <c r="AD107">
         <v>0</v>
       </c>
+      <c r="AF107">
+        <v>0</v>
+      </c>
     </row>
-    <row r="108" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="108" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A108" t="s">
         <v>30</v>
       </c>
@@ -13665,8 +13996,11 @@
       <c r="AD108">
         <v>0</v>
       </c>
+      <c r="AF108">
+        <v>0</v>
+      </c>
     </row>
-    <row r="109" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="109" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A109" t="s">
         <v>30</v>
       </c>
@@ -13754,8 +14088,11 @@
       <c r="AD109">
         <v>0</v>
       </c>
+      <c r="AF109">
+        <v>0</v>
+      </c>
     </row>
-    <row r="110" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="110" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A110" t="s">
         <v>30</v>
       </c>
@@ -13843,8 +14180,11 @@
       <c r="AD110">
         <v>0</v>
       </c>
+      <c r="AF110">
+        <v>0</v>
+      </c>
     </row>
-    <row r="111" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="111" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A111" t="s">
         <v>30</v>
       </c>
@@ -13932,8 +14272,11 @@
       <c r="AD111">
         <v>0</v>
       </c>
+      <c r="AF111">
+        <v>0</v>
+      </c>
     </row>
-    <row r="112" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="112" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A112" t="s">
         <v>30</v>
       </c>
@@ -14021,8 +14364,11 @@
       <c r="AD112">
         <v>0</v>
       </c>
+      <c r="AF112">
+        <v>0</v>
+      </c>
     </row>
-    <row r="113" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="113" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A113" t="s">
         <v>30</v>
       </c>
@@ -14110,8 +14456,11 @@
       <c r="AD113">
         <v>0</v>
       </c>
+      <c r="AF113">
+        <v>0</v>
+      </c>
     </row>
-    <row r="114" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="114" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A114" t="s">
         <v>30</v>
       </c>
@@ -14199,8 +14548,11 @@
       <c r="AD114">
         <v>0</v>
       </c>
+      <c r="AF114">
+        <v>1</v>
+      </c>
     </row>
-    <row r="115" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="115" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A115" t="s">
         <v>30</v>
       </c>
@@ -14288,8 +14640,11 @@
       <c r="AD115">
         <v>0</v>
       </c>
+      <c r="AF115">
+        <v>0</v>
+      </c>
     </row>
-    <row r="116" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="116" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A116" t="s">
         <v>30</v>
       </c>
@@ -14377,8 +14732,11 @@
       <c r="AD116">
         <v>0</v>
       </c>
+      <c r="AF116">
+        <v>0</v>
+      </c>
     </row>
-    <row r="117" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="117" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A117" t="s">
         <v>30</v>
       </c>
@@ -14469,8 +14827,11 @@
       <c r="AD117">
         <v>0</v>
       </c>
+      <c r="AF117">
+        <v>1</v>
+      </c>
     </row>
-    <row r="118" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="118" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A118" t="s">
         <v>30</v>
       </c>
@@ -14558,8 +14919,11 @@
       <c r="AD118">
         <v>0</v>
       </c>
+      <c r="AF118">
+        <v>1</v>
+      </c>
     </row>
-    <row r="119" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="119" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A119" t="s">
         <v>30</v>
       </c>
@@ -14647,8 +15011,11 @@
       <c r="AD119">
         <v>0</v>
       </c>
+      <c r="AF119">
+        <v>0</v>
+      </c>
     </row>
-    <row r="120" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="120" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A120" t="s">
         <v>30</v>
       </c>
@@ -14736,8 +15103,11 @@
       <c r="AD120">
         <v>0</v>
       </c>
+      <c r="AF120">
+        <v>0</v>
+      </c>
     </row>
-    <row r="121" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="121" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A121" t="s">
         <v>30</v>
       </c>
@@ -14825,8 +15195,11 @@
       <c r="AD121">
         <v>0</v>
       </c>
+      <c r="AF121">
+        <v>0</v>
+      </c>
     </row>
-    <row r="122" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="122" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A122" t="s">
         <v>30</v>
       </c>
@@ -14914,8 +15287,11 @@
       <c r="AD122">
         <v>0</v>
       </c>
+      <c r="AF122">
+        <v>0</v>
+      </c>
     </row>
-    <row r="123" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="123" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A123" t="s">
         <v>30</v>
       </c>
@@ -15003,8 +15379,11 @@
       <c r="AD123">
         <v>0</v>
       </c>
+      <c r="AF123">
+        <v>0</v>
+      </c>
     </row>
-    <row r="124" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="124" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A124" t="s">
         <v>30</v>
       </c>
@@ -15092,8 +15471,11 @@
       <c r="AD124">
         <v>0</v>
       </c>
+      <c r="AF124">
+        <v>0</v>
+      </c>
     </row>
-    <row r="125" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="125" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A125" t="s">
         <v>30</v>
       </c>
@@ -15181,8 +15563,11 @@
       <c r="AD125">
         <v>0</v>
       </c>
+      <c r="AF125">
+        <v>0</v>
+      </c>
     </row>
-    <row r="126" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="126" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A126" t="s">
         <v>30</v>
       </c>
@@ -15270,8 +15655,11 @@
       <c r="AD126">
         <v>0</v>
       </c>
+      <c r="AF126">
+        <v>0</v>
+      </c>
     </row>
-    <row r="127" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="127" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A127" t="s">
         <v>30</v>
       </c>
@@ -15359,8 +15747,11 @@
       <c r="AD127">
         <v>0</v>
       </c>
+      <c r="AF127">
+        <v>0</v>
+      </c>
     </row>
-    <row r="128" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="128" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A128" t="s">
         <v>30</v>
       </c>
@@ -15448,8 +15839,11 @@
       <c r="AD128">
         <v>0</v>
       </c>
+      <c r="AF128">
+        <v>0</v>
+      </c>
     </row>
-    <row r="129" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="129" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A129" t="s">
         <v>30</v>
       </c>
@@ -15537,8 +15931,11 @@
       <c r="AD129">
         <v>0</v>
       </c>
+      <c r="AF129">
+        <v>0</v>
+      </c>
     </row>
-    <row r="130" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="130" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A130" t="s">
         <v>30</v>
       </c>
@@ -15626,8 +16023,11 @@
       <c r="AD130">
         <v>0</v>
       </c>
+      <c r="AF130">
+        <v>0</v>
+      </c>
     </row>
-    <row r="131" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="131" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A131" t="s">
         <v>30</v>
       </c>
@@ -15715,8 +16115,11 @@
       <c r="AD131">
         <v>0</v>
       </c>
+      <c r="AF131">
+        <v>0</v>
+      </c>
     </row>
-    <row r="132" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="132" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A132" t="s">
         <v>30</v>
       </c>
@@ -15804,8 +16207,11 @@
       <c r="AD132">
         <v>0</v>
       </c>
+      <c r="AF132">
+        <v>0</v>
+      </c>
     </row>
-    <row r="133" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="133" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A133" t="s">
         <v>30</v>
       </c>
@@ -15893,8 +16299,11 @@
       <c r="AD133">
         <v>0</v>
       </c>
+      <c r="AF133">
+        <v>0</v>
+      </c>
     </row>
-    <row r="134" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="134" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A134" t="s">
         <v>30</v>
       </c>
@@ -15982,8 +16391,11 @@
       <c r="AD134">
         <v>0</v>
       </c>
+      <c r="AF134">
+        <v>0</v>
+      </c>
     </row>
-    <row r="135" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="135" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A135" t="s">
         <v>30</v>
       </c>
@@ -16071,8 +16483,11 @@
       <c r="AD135">
         <v>0</v>
       </c>
+      <c r="AF135">
+        <v>0</v>
+      </c>
     </row>
-    <row r="136" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="136" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A136" t="s">
         <v>30</v>
       </c>
@@ -16160,8 +16575,11 @@
       <c r="AD136">
         <v>0</v>
       </c>
+      <c r="AF136">
+        <v>0</v>
+      </c>
     </row>
-    <row r="137" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="137" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A137" t="s">
         <v>30</v>
       </c>
@@ -16252,8 +16670,11 @@
       <c r="AD137">
         <v>0</v>
       </c>
+      <c r="AF137">
+        <v>0</v>
+      </c>
     </row>
-    <row r="138" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="138" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A138" t="s">
         <v>30</v>
       </c>
@@ -16344,8 +16765,11 @@
       <c r="AD138">
         <v>0</v>
       </c>
+      <c r="AF138">
+        <v>0</v>
+      </c>
     </row>
-    <row r="139" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="139" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A139" t="s">
         <v>30</v>
       </c>
@@ -16433,8 +16857,11 @@
       <c r="AD139">
         <v>0</v>
       </c>
+      <c r="AF139">
+        <v>0</v>
+      </c>
     </row>
-    <row r="140" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="140" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A140" t="s">
         <v>30</v>
       </c>
@@ -16522,8 +16949,11 @@
       <c r="AD140">
         <v>0</v>
       </c>
+      <c r="AF140">
+        <v>0</v>
+      </c>
     </row>
-    <row r="141" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="141" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A141" t="s">
         <v>30</v>
       </c>
@@ -16611,8 +17041,11 @@
       <c r="AD141">
         <v>0</v>
       </c>
+      <c r="AF141">
+        <v>0</v>
+      </c>
     </row>
-    <row r="142" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="142" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A142" t="s">
         <v>30</v>
       </c>
@@ -16700,8 +17133,11 @@
       <c r="AD142">
         <v>0</v>
       </c>
+      <c r="AF142">
+        <v>0</v>
+      </c>
     </row>
-    <row r="143" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="143" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A143" t="s">
         <v>30</v>
       </c>
@@ -16789,8 +17225,11 @@
       <c r="AD143">
         <v>0</v>
       </c>
+      <c r="AF143">
+        <v>0</v>
+      </c>
     </row>
-    <row r="144" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="144" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A144" t="s">
         <v>30</v>
       </c>
@@ -16881,8 +17320,11 @@
       <c r="AD144">
         <v>0</v>
       </c>
+      <c r="AF144">
+        <v>0</v>
+      </c>
     </row>
-    <row r="145" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="145" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A145" t="s">
         <v>30</v>
       </c>
@@ -16970,8 +17412,11 @@
       <c r="AD145">
         <v>0</v>
       </c>
+      <c r="AF145">
+        <v>0</v>
+      </c>
     </row>
-    <row r="146" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="146" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A146" t="s">
         <v>30</v>
       </c>
@@ -17062,8 +17507,11 @@
       <c r="AD146">
         <v>0</v>
       </c>
+      <c r="AF146">
+        <v>0</v>
+      </c>
     </row>
-    <row r="147" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="147" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A147" t="s">
         <v>30</v>
       </c>
@@ -17151,8 +17599,11 @@
       <c r="AD147">
         <v>0</v>
       </c>
+      <c r="AF147">
+        <v>0</v>
+      </c>
     </row>
-    <row r="148" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="148" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A148" t="s">
         <v>30</v>
       </c>
@@ -17240,8 +17691,11 @@
       <c r="AD148">
         <v>0</v>
       </c>
+      <c r="AF148">
+        <v>0</v>
+      </c>
     </row>
-    <row r="149" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="149" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A149" t="s">
         <v>30</v>
       </c>
@@ -17329,8 +17783,11 @@
       <c r="AD149">
         <v>0</v>
       </c>
+      <c r="AF149">
+        <v>0</v>
+      </c>
     </row>
-    <row r="150" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="150" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A150" t="s">
         <v>30</v>
       </c>
@@ -17418,8 +17875,11 @@
       <c r="AD150">
         <v>0</v>
       </c>
+      <c r="AF150">
+        <v>0</v>
+      </c>
     </row>
-    <row r="151" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="151" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A151" t="s">
         <v>30</v>
       </c>
@@ -17507,8 +17967,11 @@
       <c r="AD151">
         <v>0</v>
       </c>
+      <c r="AF151">
+        <v>0</v>
+      </c>
     </row>
-    <row r="152" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="152" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A152" t="s">
         <v>30</v>
       </c>
@@ -17596,8 +18059,11 @@
       <c r="AD152">
         <v>0</v>
       </c>
+      <c r="AF152">
+        <v>1</v>
+      </c>
     </row>
-    <row r="153" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="153" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A153" t="s">
         <v>30</v>
       </c>
@@ -17685,8 +18151,11 @@
       <c r="AD153">
         <v>0</v>
       </c>
+      <c r="AF153">
+        <v>1</v>
+      </c>
     </row>
-    <row r="154" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="154" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A154" t="s">
         <v>30</v>
       </c>
@@ -17774,8 +18243,11 @@
       <c r="AD154">
         <v>0</v>
       </c>
+      <c r="AF154">
+        <v>0</v>
+      </c>
     </row>
-    <row r="155" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="155" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A155" t="s">
         <v>30</v>
       </c>
@@ -17863,8 +18335,11 @@
       <c r="AD155">
         <v>0</v>
       </c>
+      <c r="AF155">
+        <v>0</v>
+      </c>
     </row>
-    <row r="156" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="156" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A156" t="s">
         <v>30</v>
       </c>
@@ -17952,8 +18427,11 @@
       <c r="AD156">
         <v>0</v>
       </c>
+      <c r="AF156">
+        <v>0</v>
+      </c>
     </row>
-    <row r="157" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="157" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A157" t="s">
         <v>30</v>
       </c>
@@ -18044,8 +18522,11 @@
       <c r="AD157">
         <v>0</v>
       </c>
+      <c r="AF157">
+        <v>0</v>
+      </c>
     </row>
-    <row r="158" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="158" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A158" t="s">
         <v>30</v>
       </c>
@@ -18133,8 +18614,11 @@
       <c r="AD158">
         <v>0</v>
       </c>
+      <c r="AF158">
+        <v>0</v>
+      </c>
     </row>
-    <row r="159" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="159" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A159" t="s">
         <v>30</v>
       </c>
@@ -18222,8 +18706,11 @@
       <c r="AD159">
         <v>0</v>
       </c>
+      <c r="AF159">
+        <v>0</v>
+      </c>
     </row>
-    <row r="160" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="160" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A160" t="s">
         <v>30</v>
       </c>
@@ -18311,8 +18798,11 @@
       <c r="AD160">
         <v>0</v>
       </c>
+      <c r="AF160">
+        <v>0</v>
+      </c>
     </row>
-    <row r="161" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="161" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A161" t="s">
         <v>30</v>
       </c>
@@ -18400,8 +18890,11 @@
       <c r="AD161">
         <v>0</v>
       </c>
+      <c r="AF161">
+        <v>0</v>
+      </c>
     </row>
-    <row r="162" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="162" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A162" t="s">
         <v>30</v>
       </c>
@@ -18489,8 +18982,11 @@
       <c r="AD162">
         <v>0</v>
       </c>
+      <c r="AF162">
+        <v>1</v>
+      </c>
     </row>
-    <row r="163" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="163" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A163" t="s">
         <v>30</v>
       </c>
@@ -18581,8 +19077,11 @@
       <c r="AD163">
         <v>0</v>
       </c>
+      <c r="AF163">
+        <v>0</v>
+      </c>
     </row>
-    <row r="164" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="164" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A164" t="s">
         <v>30</v>
       </c>
@@ -18670,8 +19169,11 @@
       <c r="AD164">
         <v>0</v>
       </c>
+      <c r="AF164">
+        <v>0</v>
+      </c>
     </row>
-    <row r="165" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="165" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A165" t="s">
         <v>30</v>
       </c>
@@ -18759,8 +19261,11 @@
       <c r="AD165">
         <v>0</v>
       </c>
+      <c r="AF165">
+        <v>0</v>
+      </c>
     </row>
-    <row r="166" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="166" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A166" t="s">
         <v>30</v>
       </c>
@@ -18851,8 +19356,11 @@
       <c r="AD166">
         <v>0</v>
       </c>
+      <c r="AF166">
+        <v>0</v>
+      </c>
     </row>
-    <row r="167" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="167" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A167" t="s">
         <v>30</v>
       </c>
@@ -18940,8 +19448,11 @@
       <c r="AD167">
         <v>0</v>
       </c>
+      <c r="AF167">
+        <v>0</v>
+      </c>
     </row>
-    <row r="168" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="168" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A168" t="s">
         <v>30</v>
       </c>
@@ -19032,8 +19543,11 @@
       <c r="AD168">
         <v>0</v>
       </c>
+      <c r="AF168">
+        <v>0</v>
+      </c>
     </row>
-    <row r="169" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="169" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A169" t="s">
         <v>30</v>
       </c>
@@ -19121,8 +19635,11 @@
       <c r="AD169">
         <v>0</v>
       </c>
+      <c r="AF169">
+        <v>0</v>
+      </c>
     </row>
-    <row r="170" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="170" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A170" t="s">
         <v>30</v>
       </c>
@@ -19210,8 +19727,11 @@
       <c r="AD170">
         <v>0</v>
       </c>
+      <c r="AF170">
+        <v>0</v>
+      </c>
     </row>
-    <row r="171" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="171" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A171" t="s">
         <v>30</v>
       </c>
@@ -19299,8 +19819,11 @@
       <c r="AD171">
         <v>0</v>
       </c>
+      <c r="AF171">
+        <v>1</v>
+      </c>
     </row>
-    <row r="172" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="172" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A172" t="s">
         <v>30</v>
       </c>
@@ -19388,8 +19911,11 @@
       <c r="AD172">
         <v>0</v>
       </c>
+      <c r="AF172">
+        <v>0</v>
+      </c>
     </row>
-    <row r="173" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="173" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A173" t="s">
         <v>30</v>
       </c>
@@ -19480,8 +20006,11 @@
       <c r="AD173">
         <v>0</v>
       </c>
+      <c r="AF173">
+        <v>0</v>
+      </c>
     </row>
-    <row r="174" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="174" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A174" t="s">
         <v>30</v>
       </c>
@@ -19572,8 +20101,11 @@
       <c r="AD174">
         <v>0</v>
       </c>
+      <c r="AF174">
+        <v>0</v>
+      </c>
     </row>
-    <row r="175" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="175" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A175" t="s">
         <v>30</v>
       </c>
@@ -19661,8 +20193,11 @@
       <c r="AD175">
         <v>0</v>
       </c>
+      <c r="AF175">
+        <v>0</v>
+      </c>
     </row>
-    <row r="176" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="176" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A176" t="s">
         <v>30</v>
       </c>
@@ -19750,8 +20285,11 @@
       <c r="AD176">
         <v>0</v>
       </c>
+      <c r="AF176">
+        <v>0</v>
+      </c>
     </row>
-    <row r="177" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="177" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A177" t="s">
         <v>30</v>
       </c>
@@ -19842,8 +20380,11 @@
       <c r="AD177">
         <v>0</v>
       </c>
+      <c r="AF177">
+        <v>0</v>
+      </c>
     </row>
-    <row r="178" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="178" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A178" t="s">
         <v>30</v>
       </c>
@@ -19931,8 +20472,11 @@
       <c r="AD178">
         <v>0</v>
       </c>
+      <c r="AF178">
+        <v>1</v>
+      </c>
     </row>
-    <row r="179" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="179" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A179" t="s">
         <v>30</v>
       </c>
@@ -20020,8 +20564,11 @@
       <c r="AD179">
         <v>0</v>
       </c>
+      <c r="AF179">
+        <v>0</v>
+      </c>
     </row>
-    <row r="180" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="180" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A180" t="s">
         <v>30</v>
       </c>
@@ -20109,8 +20656,11 @@
       <c r="AD180">
         <v>0</v>
       </c>
+      <c r="AF180">
+        <v>0</v>
+      </c>
     </row>
-    <row r="181" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="181" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A181" t="s">
         <v>30</v>
       </c>
@@ -20198,8 +20748,11 @@
       <c r="AD181">
         <v>0</v>
       </c>
+      <c r="AF181">
+        <v>0</v>
+      </c>
     </row>
-    <row r="182" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="182" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A182" t="s">
         <v>30</v>
       </c>
@@ -20287,8 +20840,11 @@
       <c r="AD182">
         <v>0</v>
       </c>
+      <c r="AF182">
+        <v>0</v>
+      </c>
     </row>
-    <row r="183" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="183" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A183" t="s">
         <v>30</v>
       </c>
@@ -20376,8 +20932,11 @@
       <c r="AD183">
         <v>0</v>
       </c>
+      <c r="AF183">
+        <v>0</v>
+      </c>
     </row>
-    <row r="184" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="184" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A184" t="s">
         <v>30</v>
       </c>
@@ -20465,8 +21024,11 @@
       <c r="AD184">
         <v>0</v>
       </c>
+      <c r="AF184">
+        <v>0</v>
+      </c>
     </row>
-    <row r="185" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="185" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A185" t="s">
         <v>30</v>
       </c>
@@ -20557,8 +21119,11 @@
       <c r="AD185">
         <v>0</v>
       </c>
+      <c r="AF185">
+        <v>0</v>
+      </c>
     </row>
-    <row r="186" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="186" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A186" t="s">
         <v>30</v>
       </c>
@@ -20646,8 +21211,11 @@
       <c r="AD186">
         <v>0</v>
       </c>
+      <c r="AF186">
+        <v>0</v>
+      </c>
     </row>
-    <row r="187" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="187" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A187" t="s">
         <v>30</v>
       </c>
@@ -20735,8 +21303,11 @@
       <c r="AD187">
         <v>0</v>
       </c>
+      <c r="AF187">
+        <v>0</v>
+      </c>
     </row>
-    <row r="188" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="188" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A188" t="s">
         <v>30</v>
       </c>
@@ -20824,8 +21395,11 @@
       <c r="AD188">
         <v>0</v>
       </c>
+      <c r="AF188">
+        <v>0</v>
+      </c>
     </row>
-    <row r="189" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="189" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A189" t="s">
         <v>30</v>
       </c>
@@ -20913,8 +21487,11 @@
       <c r="AD189">
         <v>0</v>
       </c>
+      <c r="AF189">
+        <v>1</v>
+      </c>
     </row>
-    <row r="190" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="190" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A190" t="s">
         <v>30</v>
       </c>
@@ -21005,8 +21582,11 @@
       <c r="AD190">
         <v>0</v>
       </c>
+      <c r="AF190">
+        <v>0</v>
+      </c>
     </row>
-    <row r="191" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="191" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A191" t="s">
         <v>30</v>
       </c>
@@ -21094,8 +21674,11 @@
       <c r="AD191">
         <v>0</v>
       </c>
+      <c r="AF191">
+        <v>0</v>
+      </c>
     </row>
-    <row r="192" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="192" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A192" t="s">
         <v>30</v>
       </c>
@@ -21183,8 +21766,11 @@
       <c r="AD192">
         <v>0</v>
       </c>
+      <c r="AF192">
+        <v>0</v>
+      </c>
     </row>
-    <row r="193" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="193" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A193" t="s">
         <v>30</v>
       </c>
@@ -21272,8 +21858,11 @@
       <c r="AD193">
         <v>0</v>
       </c>
+      <c r="AF193">
+        <v>0</v>
+      </c>
     </row>
-    <row r="194" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="194" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A194" t="s">
         <v>30</v>
       </c>
@@ -21361,8 +21950,11 @@
       <c r="AD194">
         <v>0</v>
       </c>
+      <c r="AF194">
+        <v>0</v>
+      </c>
     </row>
-    <row r="195" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="195" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A195" t="s">
         <v>30</v>
       </c>
@@ -21450,8 +22042,11 @@
       <c r="AD195">
         <v>0</v>
       </c>
+      <c r="AF195">
+        <v>0</v>
+      </c>
     </row>
-    <row r="196" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="196" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A196" t="s">
         <v>30</v>
       </c>
@@ -21539,8 +22134,11 @@
       <c r="AD196">
         <v>0</v>
       </c>
+      <c r="AF196">
+        <v>0</v>
+      </c>
     </row>
-    <row r="197" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="197" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A197" t="s">
         <v>30</v>
       </c>
@@ -21628,8 +22226,11 @@
       <c r="AD197">
         <v>0</v>
       </c>
+      <c r="AF197">
+        <v>0</v>
+      </c>
     </row>
-    <row r="198" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="198" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A198" t="s">
         <v>30</v>
       </c>
@@ -21720,8 +22321,11 @@
       <c r="AD198">
         <v>0</v>
       </c>
+      <c r="AF198">
+        <v>0</v>
+      </c>
     </row>
-    <row r="199" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="199" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A199" t="s">
         <v>30</v>
       </c>
@@ -21809,8 +22413,11 @@
       <c r="AD199">
         <v>0</v>
       </c>
+      <c r="AF199">
+        <v>0</v>
+      </c>
     </row>
-    <row r="200" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="200" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A200" t="s">
         <v>30</v>
       </c>
@@ -21898,8 +22505,11 @@
       <c r="AD200">
         <v>0</v>
       </c>
+      <c r="AF200">
+        <v>0</v>
+      </c>
     </row>
-    <row r="201" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="201" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A201" t="s">
         <v>30</v>
       </c>
@@ -21987,8 +22597,11 @@
       <c r="AD201">
         <v>0</v>
       </c>
+      <c r="AF201">
+        <v>0</v>
+      </c>
     </row>
-    <row r="202" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="202" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A202" t="s">
         <v>30</v>
       </c>
@@ -22076,8 +22689,11 @@
       <c r="AD202">
         <v>0</v>
       </c>
+      <c r="AF202">
+        <v>0</v>
+      </c>
     </row>
-    <row r="203" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="203" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A203" t="s">
         <v>30</v>
       </c>
@@ -22165,8 +22781,11 @@
       <c r="AD203">
         <v>0</v>
       </c>
+      <c r="AF203">
+        <v>0</v>
+      </c>
     </row>
-    <row r="204" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="204" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A204" t="s">
         <v>30</v>
       </c>
@@ -22254,8 +22873,11 @@
       <c r="AD204">
         <v>0</v>
       </c>
+      <c r="AF204">
+        <v>0</v>
+      </c>
     </row>
-    <row r="205" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="205" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A205" t="s">
         <v>30</v>
       </c>
@@ -22343,8 +22965,11 @@
       <c r="AD205">
         <v>0</v>
       </c>
+      <c r="AF205">
+        <v>0</v>
+      </c>
     </row>
-    <row r="206" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="206" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A206" t="s">
         <v>30</v>
       </c>
@@ -22432,8 +23057,11 @@
       <c r="AD206">
         <v>0</v>
       </c>
+      <c r="AF206">
+        <v>0</v>
+      </c>
     </row>
-    <row r="207" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="207" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A207" t="s">
         <v>30</v>
       </c>
@@ -22521,8 +23149,11 @@
       <c r="AD207">
         <v>0</v>
       </c>
+      <c r="AF207">
+        <v>0</v>
+      </c>
     </row>
-    <row r="208" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="208" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A208" t="s">
         <v>30</v>
       </c>
@@ -22610,8 +23241,11 @@
       <c r="AD208">
         <v>0</v>
       </c>
+      <c r="AF208">
+        <v>0</v>
+      </c>
     </row>
-    <row r="209" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="209" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A209" t="s">
         <v>30</v>
       </c>
@@ -22699,8 +23333,11 @@
       <c r="AD209">
         <v>0</v>
       </c>
+      <c r="AF209">
+        <v>1</v>
+      </c>
     </row>
-    <row r="210" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="210" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A210" t="s">
         <v>30</v>
       </c>
@@ -22788,8 +23425,11 @@
       <c r="AD210">
         <v>0</v>
       </c>
+      <c r="AF210">
+        <v>0</v>
+      </c>
     </row>
-    <row r="211" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="211" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A211" t="s">
         <v>30</v>
       </c>
@@ -22877,8 +23517,11 @@
       <c r="AD211">
         <v>0</v>
       </c>
+      <c r="AF211">
+        <v>0</v>
+      </c>
     </row>
-    <row r="212" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="212" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A212" t="s">
         <v>30</v>
       </c>
@@ -22969,8 +23612,11 @@
       <c r="AD212">
         <v>0</v>
       </c>
+      <c r="AF212">
+        <v>0</v>
+      </c>
     </row>
-    <row r="213" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="213" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A213" t="s">
         <v>30</v>
       </c>
@@ -23058,8 +23704,11 @@
       <c r="AD213">
         <v>0</v>
       </c>
+      <c r="AF213">
+        <v>0</v>
+      </c>
     </row>
-    <row r="214" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="214" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A214" t="s">
         <v>30</v>
       </c>
@@ -23147,8 +23796,11 @@
       <c r="AD214">
         <v>0</v>
       </c>
+      <c r="AF214">
+        <v>0</v>
+      </c>
     </row>
-    <row r="215" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="215" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A215" t="s">
         <v>30</v>
       </c>
@@ -23236,8 +23888,11 @@
       <c r="AD215">
         <v>0</v>
       </c>
+      <c r="AF215">
+        <v>0</v>
+      </c>
     </row>
-    <row r="216" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="216" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A216" t="s">
         <v>30</v>
       </c>
@@ -23325,8 +23980,11 @@
       <c r="AD216">
         <v>0</v>
       </c>
+      <c r="AF216">
+        <v>0</v>
+      </c>
     </row>
-    <row r="217" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="217" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A217" t="s">
         <v>30</v>
       </c>
@@ -23417,8 +24075,11 @@
       <c r="AD217">
         <v>0</v>
       </c>
+      <c r="AF217">
+        <v>0</v>
+      </c>
     </row>
-    <row r="218" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="218" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A218" t="s">
         <v>30</v>
       </c>
@@ -23506,8 +24167,11 @@
       <c r="AD218">
         <v>0</v>
       </c>
+      <c r="AF218">
+        <v>0</v>
+      </c>
     </row>
-    <row r="219" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="219" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A219" t="s">
         <v>30</v>
       </c>
@@ -23595,8 +24259,11 @@
       <c r="AD219">
         <v>0</v>
       </c>
+      <c r="AF219">
+        <v>0</v>
+      </c>
     </row>
-    <row r="220" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="220" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A220" t="s">
         <v>30</v>
       </c>
@@ -23684,8 +24351,11 @@
       <c r="AD220">
         <v>0</v>
       </c>
+      <c r="AF220">
+        <v>0</v>
+      </c>
     </row>
-    <row r="221" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="221" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A221" t="s">
         <v>30</v>
       </c>
@@ -23773,8 +24443,11 @@
       <c r="AD221">
         <v>0</v>
       </c>
+      <c r="AF221">
+        <v>0</v>
+      </c>
     </row>
-    <row r="222" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="222" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A222" t="s">
         <v>30</v>
       </c>
@@ -23862,8 +24535,11 @@
       <c r="AD222">
         <v>0</v>
       </c>
+      <c r="AF222">
+        <v>0</v>
+      </c>
     </row>
-    <row r="223" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="223" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A223" t="s">
         <v>30</v>
       </c>
@@ -23951,8 +24627,11 @@
       <c r="AD223">
         <v>0</v>
       </c>
+      <c r="AF223">
+        <v>0</v>
+      </c>
     </row>
-    <row r="224" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="224" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A224" t="s">
         <v>30</v>
       </c>
@@ -24040,8 +24719,11 @@
       <c r="AD224">
         <v>0</v>
       </c>
+      <c r="AF224">
+        <v>0</v>
+      </c>
     </row>
-    <row r="225" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="225" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A225" t="s">
         <v>30</v>
       </c>
@@ -24129,8 +24811,11 @@
       <c r="AD225">
         <v>0</v>
       </c>
+      <c r="AF225">
+        <v>0</v>
+      </c>
     </row>
-    <row r="226" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="226" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A226" t="s">
         <v>30</v>
       </c>
@@ -24221,8 +24906,11 @@
       <c r="AD226">
         <v>0</v>
       </c>
+      <c r="AF226">
+        <v>0</v>
+      </c>
     </row>
-    <row r="227" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="227" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A227" t="s">
         <v>30</v>
       </c>
@@ -24310,8 +24998,11 @@
       <c r="AD227">
         <v>0</v>
       </c>
+      <c r="AF227">
+        <v>1</v>
+      </c>
     </row>
-    <row r="228" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="228" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A228" t="s">
         <v>30</v>
       </c>
@@ -24399,8 +25090,11 @@
       <c r="AD228">
         <v>0</v>
       </c>
+      <c r="AF228">
+        <v>1</v>
+      </c>
     </row>
-    <row r="229" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="229" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A229" t="s">
         <v>30</v>
       </c>
@@ -24488,8 +25182,11 @@
       <c r="AD229">
         <v>0</v>
       </c>
+      <c r="AF229">
+        <v>0</v>
+      </c>
     </row>
-    <row r="230" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="230" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A230" t="s">
         <v>30</v>
       </c>
@@ -24577,8 +25274,11 @@
       <c r="AD230">
         <v>0</v>
       </c>
+      <c r="AF230">
+        <v>0</v>
+      </c>
     </row>
-    <row r="231" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="231" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A231" t="s">
         <v>30</v>
       </c>
@@ -24666,8 +25366,11 @@
       <c r="AD231">
         <v>0</v>
       </c>
+      <c r="AF231">
+        <v>1</v>
+      </c>
     </row>
-    <row r="232" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="232" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A232" t="s">
         <v>30</v>
       </c>
@@ -24758,8 +25461,11 @@
       <c r="AD232">
         <v>0</v>
       </c>
+      <c r="AF232">
+        <v>0</v>
+      </c>
     </row>
-    <row r="233" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="233" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A233" t="s">
         <v>30</v>
       </c>
@@ -24847,8 +25553,11 @@
       <c r="AD233">
         <v>0</v>
       </c>
+      <c r="AF233">
+        <v>0</v>
+      </c>
     </row>
-    <row r="234" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="234" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A234" t="s">
         <v>30</v>
       </c>
@@ -24936,8 +25645,11 @@
       <c r="AD234">
         <v>0</v>
       </c>
+      <c r="AF234">
+        <v>0</v>
+      </c>
     </row>
-    <row r="235" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="235" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A235" t="s">
         <v>30</v>
       </c>
@@ -25025,8 +25737,11 @@
       <c r="AD235">
         <v>0</v>
       </c>
+      <c r="AF235">
+        <v>0</v>
+      </c>
     </row>
-    <row r="236" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="236" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A236" t="s">
         <v>30</v>
       </c>
@@ -25114,8 +25829,11 @@
       <c r="AD236">
         <v>0</v>
       </c>
+      <c r="AF236">
+        <v>0</v>
+      </c>
     </row>
-    <row r="237" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="237" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A237" t="s">
         <v>30</v>
       </c>
@@ -25203,8 +25921,11 @@
       <c r="AD237">
         <v>0</v>
       </c>
+      <c r="AF237">
+        <v>0</v>
+      </c>
     </row>
-    <row r="238" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="238" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A238" t="s">
         <v>30</v>
       </c>
@@ -25292,8 +26013,11 @@
       <c r="AD238">
         <v>0</v>
       </c>
+      <c r="AF238">
+        <v>0</v>
+      </c>
     </row>
-    <row r="239" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="239" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A239" t="s">
         <v>30</v>
       </c>
@@ -25378,8 +26102,11 @@
       <c r="AD239">
         <v>0</v>
       </c>
+      <c r="AF239">
+        <v>0</v>
+      </c>
     </row>
-    <row r="240" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="240" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A240" t="s">
         <v>30</v>
       </c>
@@ -25467,8 +26194,11 @@
       <c r="AD240">
         <v>0</v>
       </c>
+      <c r="AF240">
+        <v>0</v>
+      </c>
     </row>
-    <row r="241" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="241" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A241" t="s">
         <v>30</v>
       </c>
@@ -25556,8 +26286,11 @@
       <c r="AD241">
         <v>0</v>
       </c>
+      <c r="AF241">
+        <v>1</v>
+      </c>
     </row>
-    <row r="242" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="242" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A242" t="s">
         <v>30</v>
       </c>
@@ -25645,8 +26378,11 @@
       <c r="AD242">
         <v>0</v>
       </c>
+      <c r="AF242">
+        <v>0</v>
+      </c>
     </row>
-    <row r="243" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="243" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A243" t="s">
         <v>30</v>
       </c>
@@ -25734,8 +26470,11 @@
       <c r="AD243">
         <v>0</v>
       </c>
+      <c r="AF243">
+        <v>0</v>
+      </c>
     </row>
-    <row r="244" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="244" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A244" t="s">
         <v>30</v>
       </c>
@@ -25823,8 +26562,11 @@
       <c r="AD244">
         <v>0</v>
       </c>
+      <c r="AF244">
+        <v>1</v>
+      </c>
     </row>
-    <row r="245" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="245" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A245" t="s">
         <v>30</v>
       </c>
@@ -25912,8 +26654,11 @@
       <c r="AD245">
         <v>0</v>
       </c>
+      <c r="AF245">
+        <v>0</v>
+      </c>
     </row>
-    <row r="246" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="246" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A246" t="s">
         <v>30</v>
       </c>
@@ -26001,8 +26746,11 @@
       <c r="AD246">
         <v>0</v>
       </c>
+      <c r="AF246">
+        <v>0</v>
+      </c>
     </row>
-    <row r="247" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="247" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A247" t="s">
         <v>30</v>
       </c>
@@ -26090,8 +26838,11 @@
       <c r="AD247">
         <v>0</v>
       </c>
+      <c r="AF247">
+        <v>0</v>
+      </c>
     </row>
-    <row r="248" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="248" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A248" t="s">
         <v>30</v>
       </c>
@@ -26179,8 +26930,11 @@
       <c r="AD248">
         <v>0</v>
       </c>
+      <c r="AF248">
+        <v>0</v>
+      </c>
     </row>
-    <row r="249" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="249" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A249" t="s">
         <v>30</v>
       </c>
@@ -26268,8 +27022,11 @@
       <c r="AD249">
         <v>0</v>
       </c>
+      <c r="AF249">
+        <v>0</v>
+      </c>
     </row>
-    <row r="250" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="250" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A250" t="s">
         <v>30</v>
       </c>
@@ -26357,8 +27114,11 @@
       <c r="AD250">
         <v>0</v>
       </c>
+      <c r="AF250">
+        <v>0</v>
+      </c>
     </row>
-    <row r="251" spans="1:30" x14ac:dyDescent="0.35">
+    <row r="251" spans="1:32" x14ac:dyDescent="0.3">
       <c r="A251" t="s">
         <v>30</v>
       </c>
@@ -26446,9 +27206,11 @@
       <c r="AD251">
         <v>0</v>
       </c>
+      <c r="AF251">
+        <v>1</v>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:AD251" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>